<commit_message>
Update Excel file via delegated auth - Wed Oct 21 13:27:36 UTC 2026
</commit_message>
<xml_diff>
--- a/data/Extra Grants_latest.xlsx
+++ b/data/Extra Grants_latest.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30516"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30611"/>
   <workbookPr codeName="ThisWorkbook" hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aphrcorg-my.sharepoint.com/personal/nnjenga_aphrc_org/Documents/CARTA Dashboard/ECRS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="509" documentId="13_ncr:1_{D015934C-5C8D-463B-9777-448ADC1EE7B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{33C916BA-8656-4457-A29D-220595C8E40E}"/>
+  <xr:revisionPtr revIDLastSave="512" documentId="13_ncr:1_{D015934C-5C8D-463B-9777-448ADC1EE7B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1AD65A88-CF7B-4379-88D6-88A30F94ED34}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
   </definedNames>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="29" r:id="rId7"/>
+    <pivotCache cacheId="317" r:id="rId7"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -6327,36 +6327,6 @@
       <numFmt numFmtId="166" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="169" formatCode="_-* #,##0.0_-;\-* #,##0.0_-;_-* &quot;-&quot;??_-;_-@_-"/>
     </dxf>
     <dxf>
@@ -6394,6 +6364,36 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="166" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="166" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
@@ -14800,6 +14800,9 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
       <x14:pivotCacheDefinition/>
     </ext>
+    <ext xmlns:xlpdsc="http://schemas.microsoft.com/office/spreadsheetml/2026/pivotDataSourceClean" uri="{F4336242-56EE-4DD3-A5F7-E900642BF6E9}">
+      <xlpdsc:dataSourceClean>1</xlpdsc:dataSourceClean>
+    </ext>
   </extLst>
 </pivotCacheDefinition>
 </file>
@@ -28310,7 +28313,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{551C2CDB-7398-421C-88CA-55BBA8F543FA}" name="PivotTable1" cacheId="29" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{551C2CDB-7398-421C-88CA-55BBA8F543FA}" name="PivotTable1" cacheId="317" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A5:E149" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="3" colPageCount="1"/>
   <pivotFields count="25">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -29033,46 +29036,46 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable10.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8AF8FCFC-489E-4F8D-895C-35AB7CBDA56C}" name="PivotTable11" cacheId="29" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" showMissing="0" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="13">
-  <location ref="B50:F63" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="4" colPageCount="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000002000000}" name="PivotTable3" cacheId="317" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" showMissing="0" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="3">
+  <location ref="B7:E11" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="4" colPageCount="1"/>
   <pivotFields count="25">
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField axis="axisPage" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
       <items count="35">
-        <item x="1"/>
-        <item x="4"/>
-        <item x="12"/>
-        <item x="6"/>
-        <item x="18"/>
-        <item x="23"/>
-        <item x="3"/>
-        <item x="2"/>
-        <item x="5"/>
-        <item x="14"/>
-        <item x="20"/>
-        <item x="8"/>
-        <item x="11"/>
-        <item x="17"/>
+        <item h="1" x="1"/>
+        <item h="1" x="4"/>
+        <item h="1" x="12"/>
+        <item h="1" x="6"/>
+        <item h="1" x="18"/>
+        <item h="1" x="23"/>
+        <item h="1" x="3"/>
+        <item h="1" x="2"/>
+        <item h="1" x="5"/>
+        <item h="1" x="14"/>
+        <item h="1" x="20"/>
+        <item h="1" x="8"/>
+        <item h="1" x="11"/>
+        <item h="1" x="17"/>
         <item m="1" x="33"/>
-        <item x="9"/>
-        <item x="13"/>
-        <item x="19"/>
-        <item x="10"/>
-        <item x="15"/>
-        <item x="22"/>
-        <item x="7"/>
-        <item x="16"/>
-        <item x="21"/>
-        <item x="0"/>
-        <item x="24"/>
-        <item m="1" x="32"/>
-        <item x="25"/>
-        <item x="26"/>
-        <item x="27"/>
+        <item h="1" x="9"/>
+        <item h="1" x="13"/>
+        <item h="1" x="19"/>
+        <item h="1" x="10"/>
+        <item h="1" x="15"/>
+        <item h="1" x="22"/>
+        <item h="1" x="7"/>
+        <item h="1" x="16"/>
+        <item h="1" x="21"/>
+        <item h="1" x="0"/>
+        <item h="1" x="24"/>
+        <item h="1" m="1" x="32"/>
+        <item h="1" x="25"/>
+        <item h="1" x="26"/>
+        <item h="1" x="27"/>
         <item x="29"/>
         <item x="28"/>
-        <item x="30"/>
-        <item x="31"/>
+        <item h="1" x="30"/>
+        <item h="1" x="31"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -29195,39 +29198,12 @@
   <rowFields count="1">
     <field x="16"/>
   </rowFields>
-  <rowItems count="12">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
+  <rowItems count="3">
     <i>
       <x v="8"/>
     </i>
     <i>
       <x v="9"/>
-    </i>
-    <i>
-      <x v="10"/>
     </i>
     <i t="grand">
       <x/>
@@ -29236,15 +29212,12 @@
   <colFields count="1">
     <field x="6"/>
   </colFields>
-  <colItems count="4">
+  <colItems count="3">
     <i>
       <x/>
     </i>
     <i>
       <x v="1"/>
-    </i>
-    <i>
-      <x v="3"/>
     </i>
     <i t="grand">
       <x/>
@@ -29257,7 +29230,7 @@
     <pageField fld="10" hier="-1"/>
   </pageFields>
   <dataFields count="1">
-    <dataField name="Sum of Total amount in $" fld="12" baseField="16" baseItem="4"/>
+    <dataField name="Count of Total amount in $" fld="12" subtotal="count" baseField="16" baseItem="0" numFmtId="166"/>
   </dataFields>
   <formats count="2">
     <format dxfId="34">
@@ -29267,8 +29240,8 @@
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
-  <conditionalFormats count="2">
-    <conditionalFormat priority="4">
+  <conditionalFormats count="1">
+    <conditionalFormat priority="6">
       <pivotAreas count="1">
         <pivotArea type="data" collapsedLevelsAreSubtotals="1" fieldPosition="0">
           <references count="2">
@@ -29286,25 +29259,8 @@
         </pivotArea>
       </pivotAreas>
     </conditionalFormat>
-    <conditionalFormat priority="3">
-      <pivotAreas count="1">
-        <pivotArea type="data" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
-          <references count="2">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-            <reference field="16" count="4" selected="0">
-              <x v="6"/>
-              <x v="7"/>
-              <x v="8"/>
-              <x v="9"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </pivotAreas>
-    </conditionalFormat>
   </conditionalFormats>
-  <chartFormats count="13">
+  <chartFormats count="4">
     <chartFormat chart="2" format="6" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="2">
@@ -29353,114 +29309,6 @@
         </references>
       </pivotArea>
     </chartFormat>
-    <chartFormat chart="6" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="6" format="1" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="6" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="3"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="9" format="6" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="9" format="7" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="9" format="8" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="3"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="12" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="12" format="1" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="12" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="3"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
   </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
@@ -29475,7 +29323,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable11.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000003000000}" name="PivotTable4" cacheId="29" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" showMissing="0" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000003000000}" name="PivotTable4" cacheId="317" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" showMissing="0" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="B5:F39" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="25">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -29730,7 +29578,283 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000005000000}" name="PivotTable6" cacheId="29" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" showMissing="0" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable1" cacheId="317" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" showMissing="0" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+  <location ref="A55:E68" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="3" colPageCount="1"/>
+  <pivotFields count="25">
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField axis="axisCol" compact="0" outline="0" showAll="0">
+      <items count="5">
+        <item x="2"/>
+        <item x="1"/>
+        <item m="1" x="3"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisPage" compact="0" outline="0" showAll="0">
+      <items count="15">
+        <item x="5"/>
+        <item x="9"/>
+        <item x="6"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="10"/>
+        <item m="1" x="13"/>
+        <item x="0"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField axis="axisPage" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
+      <items count="35">
+        <item m="1" x="29"/>
+        <item x="1"/>
+        <item m="1" x="30"/>
+        <item m="1" x="31"/>
+        <item m="1" x="24"/>
+        <item x="6"/>
+        <item x="5"/>
+        <item m="1" x="27"/>
+        <item m="1" x="23"/>
+        <item m="1" x="32"/>
+        <item m="1" x="21"/>
+        <item m="1" x="25"/>
+        <item x="3"/>
+        <item x="7"/>
+        <item x="20"/>
+        <item x="2"/>
+        <item m="1" x="28"/>
+        <item m="1" x="26"/>
+        <item m="1" x="22"/>
+        <item x="4"/>
+        <item x="8"/>
+        <item m="1" x="33"/>
+        <item x="0"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField dataField="1" compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0">
+      <items count="12">
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField axis="axisPage" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
+      <items count="10">
+        <item x="2"/>
+        <item x="1"/>
+        <item x="0"/>
+        <item h="1" m="1" x="7"/>
+        <item h="1" m="1" x="8"/>
+        <item h="1" m="1" x="3"/>
+        <item h="1" m="1" x="4"/>
+        <item h="1" m="1" x="5"/>
+        <item h="1" m="1" x="6"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="16"/>
+  </rowFields>
+  <rowItems count="12">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="6"/>
+  </colFields>
+  <colItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <pageFields count="3">
+    <pageField fld="7" hier="-1"/>
+    <pageField fld="18" hier="-1"/>
+    <pageField fld="10" hier="-1"/>
+  </pageFields>
+  <dataFields count="1">
+    <dataField name="Count of Total amount in $" fld="12" subtotal="count" baseField="16" baseItem="2" numFmtId="1"/>
+  </dataFields>
+  <formats count="10">
+    <format dxfId="55">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="56">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="57">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="58">
+      <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="59">
+      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="60">
+      <pivotArea field="16" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="61">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="16" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="62">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="63">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="6" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="64">
+      <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
+    </format>
+  </formats>
+  <conditionalFormats count="2">
+    <conditionalFormat priority="10">
+      <pivotAreas count="1">
+        <pivotArea type="data" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="16" count="5">
+              <x v="0"/>
+              <x v="1"/>
+              <x v="2"/>
+              <x v="3"/>
+              <x v="4"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </pivotAreas>
+    </conditionalFormat>
+    <conditionalFormat priority="5">
+      <pivotAreas count="1">
+        <pivotArea type="data" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="16" count="3" selected="0">
+              <x v="5"/>
+              <x v="6"/>
+              <x v="7"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </pivotAreas>
+    </conditionalFormat>
+  </conditionalFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000005000000}" name="PivotTable6" cacheId="317" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" showMissing="0" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A27:E29" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="25">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -29817,7 +29941,7 @@
     <dataField name="Sum of Total amount in $" fld="12" baseField="8" baseItem="5" numFmtId="166"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="64">
+    <format dxfId="54">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -29833,8 +29957,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2B407599-BB24-4523-B687-82A24A40E00E}" name="PivotTable3" cacheId="29" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" showMissing="0" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="7">
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2B407599-BB24-4523-B687-82A24A40E00E}" name="PivotTable3" cacheId="317" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" showMissing="0" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="7">
   <location ref="A141:E156" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="25">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -29983,7 +30107,7 @@
     <dataField name="Sum of Total amount in $" fld="12" baseField="8" baseItem="5" numFmtId="166"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="63">
+    <format dxfId="53">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -30037,8 +30161,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000001000000}" name="PivotTable2" cacheId="29" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" showMissing="0" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000001000000}" name="PivotTable2" cacheId="317" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" showMissing="0" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A82:B134" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="4" colPageCount="1"/>
   <pivotFields count="25">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -30479,35 +30603,35 @@
     <dataField name="Sum of Total amount in $" fld="12" baseField="2" baseItem="5"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="54">
+    <format dxfId="44">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="55">
+    <format dxfId="45">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="56">
+    <format dxfId="46">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="57">
+    <format dxfId="47">
       <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0"/>
     </format>
-    <format dxfId="58">
+    <format dxfId="48">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="59">
+    <format dxfId="49">
       <pivotArea field="16" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisPage" fieldPosition="0"/>
     </format>
-    <format dxfId="60">
+    <format dxfId="50">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="16" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="61">
+    <format dxfId="51">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="62">
+    <format dxfId="52">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -30523,8 +30647,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000004000000}" name="PivotTable5" cacheId="29" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" showMissing="0" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="10">
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000004000000}" name="PivotTable5" cacheId="317" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" showMissing="0" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="10">
   <location ref="A6:E19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="4" colPageCount="1"/>
   <pivotFields count="25">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -30751,14 +30875,29 @@
     <dataField name="Sum of Total amount in $" fld="12" baseField="16" baseItem="4"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="52">
+    <format dxfId="42">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="53">
+    <format dxfId="43">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
   <conditionalFormats count="2">
+    <conditionalFormat priority="1">
+      <pivotAreas count="1">
+        <pivotArea type="data" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="16" count="2" selected="0">
+              <x v="9"/>
+              <x v="10"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </pivotAreas>
+    </conditionalFormat>
     <conditionalFormat priority="4">
       <pivotAreas count="1">
         <pivotArea type="data" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
@@ -30776,21 +30915,6 @@
               <x v="6"/>
               <x v="7"/>
               <x v="8"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </pivotAreas>
-    </conditionalFormat>
-    <conditionalFormat priority="1">
-      <pivotAreas count="1">
-        <pivotArea type="data" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
-          <references count="2">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-            <reference field="16" count="2" selected="0">
-              <x v="9"/>
-              <x v="10"/>
             </reference>
           </references>
         </pivotArea>
@@ -30886,12 +31010,432 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable1" cacheId="29" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" showMissing="0" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
-  <location ref="A55:E68" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="3" colPageCount="1"/>
+<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{518325C7-055A-4FD7-8A8B-DEB66D95FD13}" name="PivotTable1" cacheId="317" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" showMissing="0" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="22">
+  <location ref="B74:C78" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="4" colPageCount="1"/>
   <pivotFields count="25">
     <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField axis="axisPage" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
+      <items count="35">
+        <item x="1"/>
+        <item x="4"/>
+        <item x="12"/>
+        <item x="6"/>
+        <item x="18"/>
+        <item x="23"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item x="5"/>
+        <item x="14"/>
+        <item x="20"/>
+        <item x="8"/>
+        <item x="11"/>
+        <item x="17"/>
+        <item m="1" x="33"/>
+        <item x="9"/>
+        <item x="13"/>
+        <item x="19"/>
+        <item x="10"/>
+        <item x="15"/>
+        <item x="22"/>
+        <item x="7"/>
+        <item x="16"/>
+        <item x="21"/>
+        <item x="0"/>
+        <item x="24"/>
+        <item m="1" x="32"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="29"/>
+        <item x="28"/>
+        <item x="30"/>
+        <item x="31"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0">
+      <items count="5">
+        <item x="2"/>
+        <item x="1"/>
+        <item m="1" x="3"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisPage" compact="0" outline="0" showAll="0">
+      <items count="15">
+        <item x="5"/>
+        <item x="9"/>
+        <item x="6"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="10"/>
+        <item m="1" x="13"/>
+        <item x="0"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField axis="axisPage" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
+      <items count="35">
+        <item m="1" x="29"/>
+        <item x="1"/>
+        <item m="1" x="30"/>
+        <item m="1" x="31"/>
+        <item m="1" x="24"/>
+        <item x="6"/>
+        <item x="5"/>
+        <item m="1" x="27"/>
+        <item m="1" x="23"/>
+        <item m="1" x="32"/>
+        <item m="1" x="21"/>
+        <item m="1" x="25"/>
+        <item x="3"/>
+        <item x="7"/>
+        <item x="20"/>
+        <item x="2"/>
+        <item m="1" x="28"/>
+        <item m="1" x="26"/>
+        <item m="1" x="22"/>
+        <item x="4"/>
+        <item x="8"/>
+        <item m="1" x="33"/>
+        <item x="0"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField dataField="1" compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0" sortType="ascending"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField axis="axisPage" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
+      <items count="10">
+        <item x="2"/>
+        <item x="1"/>
+        <item x="0"/>
+        <item m="1" x="7"/>
+        <item m="1" x="8"/>
+        <item m="1" x="3"/>
+        <item m="1" x="4"/>
+        <item m="1" x="5"/>
+        <item m="1" x="6"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="6"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <pageFields count="4">
+    <pageField fld="7" hier="-1"/>
+    <pageField fld="1" hier="-1"/>
+    <pageField fld="18" hier="-1"/>
+    <pageField fld="10" hier="-1"/>
+  </pageFields>
+  <dataFields count="1">
+    <dataField name="Sum of Total amount in $" fld="12" baseField="16" baseItem="4"/>
+  </dataFields>
+  <formats count="2">
+    <format dxfId="40">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="41">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="16">
+    <chartFormat chart="2" format="6" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="7" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="8" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="9" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="6" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="6" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="6" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="9" format="6" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="9" format="7" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="9" format="8" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="12" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="12" format="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="17" format="6" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="17" format="7">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="17" format="8">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="17" format="9">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8AF8FCFC-489E-4F8D-895C-35AB7CBDA56C}" name="PivotTable11" cacheId="317" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" showMissing="0" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="13">
+  <location ref="B50:F63" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="4" colPageCount="1"/>
+  <pivotFields count="25">
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField axis="axisPage" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
+      <items count="35">
+        <item x="1"/>
+        <item x="4"/>
+        <item x="12"/>
+        <item x="6"/>
+        <item x="18"/>
+        <item x="23"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item x="5"/>
+        <item x="14"/>
+        <item x="20"/>
+        <item x="8"/>
+        <item x="11"/>
+        <item x="17"/>
+        <item m="1" x="33"/>
+        <item x="9"/>
+        <item x="13"/>
+        <item x="19"/>
+        <item x="10"/>
+        <item x="15"/>
+        <item x="22"/>
+        <item x="7"/>
+        <item x="16"/>
+        <item x="21"/>
+        <item x="0"/>
+        <item x="24"/>
+        <item m="1" x="32"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="29"/>
+        <item x="28"/>
+        <item x="30"/>
+        <item x="31"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -30970,14 +31514,14 @@
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField axis="axisRow" compact="0" outline="0" showAll="0">
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" sortType="ascending">
       <items count="12">
+        <item x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
         <item x="4"/>
         <item x="5"/>
-        <item x="0"/>
         <item x="6"/>
         <item x="7"/>
         <item x="8"/>
@@ -30992,12 +31536,12 @@
         <item x="2"/>
         <item x="1"/>
         <item x="0"/>
-        <item h="1" m="1" x="7"/>
-        <item h="1" m="1" x="8"/>
-        <item h="1" m="1" x="3"/>
-        <item h="1" m="1" x="4"/>
-        <item h="1" m="1" x="5"/>
-        <item h="1" m="1" x="6"/>
+        <item m="1" x="7"/>
+        <item m="1" x="8"/>
+        <item m="1" x="3"/>
+        <item m="1" x="4"/>
+        <item m="1" x="5"/>
+        <item m="1" x="6"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -31066,72 +31610,42 @@
       <x/>
     </i>
   </colItems>
-  <pageFields count="3">
+  <pageFields count="4">
     <pageField fld="7" hier="-1"/>
+    <pageField fld="1" hier="-1"/>
     <pageField fld="18" hier="-1"/>
     <pageField fld="10" hier="-1"/>
   </pageFields>
   <dataFields count="1">
-    <dataField name="Count of Total amount in $" fld="12" subtotal="count" baseField="16" baseItem="2" numFmtId="1"/>
+    <dataField name="Sum of Total amount in $" fld="12" baseField="16" baseItem="4"/>
   </dataFields>
-  <formats count="10">
-    <format dxfId="42">
-      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="43">
+  <formats count="2">
+    <format dxfId="38">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="44">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="45">
-      <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
-    </format>
-    <format dxfId="46">
-      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="47">
-      <pivotArea field="16" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="48">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="16" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="49">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="50">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="6" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="51">
-      <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
+    <format dxfId="39">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
   <conditionalFormats count="2">
-    <conditionalFormat priority="5">
+    <conditionalFormat priority="3">
       <pivotAreas count="1">
         <pivotArea type="data" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
           <references count="2">
             <reference field="4294967294" count="1" selected="0">
               <x v="0"/>
             </reference>
-            <reference field="16" count="3" selected="0">
-              <x v="5"/>
+            <reference field="16" count="4" selected="0">
               <x v="6"/>
               <x v="7"/>
+              <x v="8"/>
+              <x v="9"/>
             </reference>
           </references>
         </pivotArea>
       </pivotAreas>
     </conditionalFormat>
-    <conditionalFormat priority="10">
+    <conditionalFormat priority="4">
       <pivotAreas count="1">
         <pivotArea type="data" collapsedLevelsAreSubtotals="1" fieldPosition="0">
           <references count="2">
@@ -31139,17 +31653,175 @@
               <x v="0"/>
             </reference>
             <reference field="16" count="5">
-              <x v="0"/>
               <x v="1"/>
               <x v="2"/>
               <x v="3"/>
               <x v="4"/>
+              <x v="5"/>
             </reference>
           </references>
         </pivotArea>
       </pivotAreas>
     </conditionalFormat>
   </conditionalFormats>
+  <chartFormats count="13">
+    <chartFormat chart="2" format="6" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="7" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="8" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="9" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="6" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="6" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="6" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="9" format="6" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="9" format="7" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="9" format="8" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="12" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="12" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="12" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -31162,8 +31834,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0325BBC9-6471-430A-8157-D1A40160D7A8}" name="PivotTable10" cacheId="29" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" showMissing="0" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="3">
+<file path=xl/pivotTables/pivotTable9.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0325BBC9-6471-430A-8157-D1A40160D7A8}" name="PivotTable10" cacheId="317" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" showMissing="0" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="3">
   <location ref="B28:E40" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="4" colPageCount="1"/>
   <pivotFields count="25">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -31384,10 +32056,10 @@
     <dataField name="Sum of Total amount in $" fld="12" baseField="16" baseItem="4"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="40">
+    <format dxfId="36">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="41">
+    <format dxfId="37">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -31473,683 +32145,9 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000002000000}" name="PivotTable3" cacheId="29" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" showMissing="0" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="3">
-  <location ref="B7:E11" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="4" colPageCount="1"/>
-  <pivotFields count="25">
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField axis="axisPage" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
-      <items count="35">
-        <item h="1" x="1"/>
-        <item h="1" x="4"/>
-        <item h="1" x="12"/>
-        <item h="1" x="6"/>
-        <item h="1" x="18"/>
-        <item h="1" x="23"/>
-        <item h="1" x="3"/>
-        <item h="1" x="2"/>
-        <item h="1" x="5"/>
-        <item h="1" x="14"/>
-        <item h="1" x="20"/>
-        <item h="1" x="8"/>
-        <item h="1" x="11"/>
-        <item h="1" x="17"/>
-        <item m="1" x="33"/>
-        <item h="1" x="9"/>
-        <item h="1" x="13"/>
-        <item h="1" x="19"/>
-        <item h="1" x="10"/>
-        <item h="1" x="15"/>
-        <item h="1" x="22"/>
-        <item h="1" x="7"/>
-        <item h="1" x="16"/>
-        <item h="1" x="21"/>
-        <item h="1" x="0"/>
-        <item h="1" x="24"/>
-        <item h="1" m="1" x="32"/>
-        <item h="1" x="25"/>
-        <item h="1" x="26"/>
-        <item h="1" x="27"/>
-        <item x="29"/>
-        <item x="28"/>
-        <item h="1" x="30"/>
-        <item h="1" x="31"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField axis="axisCol" compact="0" outline="0" showAll="0">
-      <items count="5">
-        <item x="2"/>
-        <item x="1"/>
-        <item m="1" x="3"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisPage" compact="0" outline="0" showAll="0">
-      <items count="15">
-        <item x="5"/>
-        <item x="9"/>
-        <item x="6"/>
-        <item x="1"/>
-        <item x="4"/>
-        <item x="3"/>
-        <item x="2"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="10"/>
-        <item m="1" x="13"/>
-        <item x="0"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField axis="axisPage" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
-      <items count="35">
-        <item m="1" x="29"/>
-        <item x="1"/>
-        <item m="1" x="30"/>
-        <item m="1" x="31"/>
-        <item m="1" x="24"/>
-        <item x="6"/>
-        <item x="5"/>
-        <item m="1" x="27"/>
-        <item m="1" x="23"/>
-        <item m="1" x="32"/>
-        <item m="1" x="21"/>
-        <item m="1" x="25"/>
-        <item x="3"/>
-        <item x="7"/>
-        <item x="20"/>
-        <item x="2"/>
-        <item m="1" x="28"/>
-        <item m="1" x="26"/>
-        <item m="1" x="22"/>
-        <item x="4"/>
-        <item x="8"/>
-        <item m="1" x="33"/>
-        <item x="0"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item x="14"/>
-        <item x="15"/>
-        <item x="16"/>
-        <item x="17"/>
-        <item x="18"/>
-        <item x="19"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField dataField="1" compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" sortType="ascending">
-      <items count="12">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField axis="axisPage" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
-      <items count="10">
-        <item x="2"/>
-        <item x="1"/>
-        <item x="0"/>
-        <item m="1" x="7"/>
-        <item m="1" x="8"/>
-        <item m="1" x="3"/>
-        <item m="1" x="4"/>
-        <item m="1" x="5"/>
-        <item m="1" x="6"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="16"/>
-  </rowFields>
-  <rowItems count="3">
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="6"/>
-  </colFields>
-  <colItems count="3">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <pageFields count="4">
-    <pageField fld="7" hier="-1"/>
-    <pageField fld="1" hier="-1"/>
-    <pageField fld="18" hier="-1"/>
-    <pageField fld="10" hier="-1"/>
-  </pageFields>
-  <dataFields count="1">
-    <dataField name="Count of Total amount in $" fld="12" subtotal="count" baseField="16" baseItem="0" numFmtId="166"/>
-  </dataFields>
-  <formats count="2">
-    <format dxfId="38">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="39">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-  </formats>
-  <conditionalFormats count="1">
-    <conditionalFormat priority="6">
-      <pivotAreas count="1">
-        <pivotArea type="data" collapsedLevelsAreSubtotals="1" fieldPosition="0">
-          <references count="2">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-            <reference field="16" count="5">
-              <x v="1"/>
-              <x v="2"/>
-              <x v="3"/>
-              <x v="4"/>
-              <x v="5"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </pivotAreas>
-    </conditionalFormat>
-  </conditionalFormats>
-  <chartFormats count="4">
-    <chartFormat chart="2" format="6" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="2" format="7" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="2" format="8" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="3"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="2" format="9" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable9.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{518325C7-055A-4FD7-8A8B-DEB66D95FD13}" name="PivotTable1" cacheId="29" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" showMissing="0" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="22">
-  <location ref="B74:C78" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="4" colPageCount="1"/>
-  <pivotFields count="25">
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField axis="axisPage" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
-      <items count="35">
-        <item x="1"/>
-        <item x="4"/>
-        <item x="12"/>
-        <item x="6"/>
-        <item x="18"/>
-        <item x="23"/>
-        <item x="3"/>
-        <item x="2"/>
-        <item x="5"/>
-        <item x="14"/>
-        <item x="20"/>
-        <item x="8"/>
-        <item x="11"/>
-        <item x="17"/>
-        <item m="1" x="33"/>
-        <item x="9"/>
-        <item x="13"/>
-        <item x="19"/>
-        <item x="10"/>
-        <item x="15"/>
-        <item x="22"/>
-        <item x="7"/>
-        <item x="16"/>
-        <item x="21"/>
-        <item x="0"/>
-        <item x="24"/>
-        <item m="1" x="32"/>
-        <item x="25"/>
-        <item x="26"/>
-        <item x="27"/>
-        <item x="29"/>
-        <item x="28"/>
-        <item x="30"/>
-        <item x="31"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField axis="axisRow" compact="0" outline="0" showAll="0">
-      <items count="5">
-        <item x="2"/>
-        <item x="1"/>
-        <item m="1" x="3"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisPage" compact="0" outline="0" showAll="0">
-      <items count="15">
-        <item x="5"/>
-        <item x="9"/>
-        <item x="6"/>
-        <item x="1"/>
-        <item x="4"/>
-        <item x="3"/>
-        <item x="2"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="10"/>
-        <item m="1" x="13"/>
-        <item x="0"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField axis="axisPage" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
-      <items count="35">
-        <item m="1" x="29"/>
-        <item x="1"/>
-        <item m="1" x="30"/>
-        <item m="1" x="31"/>
-        <item m="1" x="24"/>
-        <item x="6"/>
-        <item x="5"/>
-        <item m="1" x="27"/>
-        <item m="1" x="23"/>
-        <item m="1" x="32"/>
-        <item m="1" x="21"/>
-        <item m="1" x="25"/>
-        <item x="3"/>
-        <item x="7"/>
-        <item x="20"/>
-        <item x="2"/>
-        <item m="1" x="28"/>
-        <item m="1" x="26"/>
-        <item m="1" x="22"/>
-        <item x="4"/>
-        <item x="8"/>
-        <item m="1" x="33"/>
-        <item x="0"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item x="14"/>
-        <item x="15"/>
-        <item x="16"/>
-        <item x="17"/>
-        <item x="18"/>
-        <item x="19"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField dataField="1" compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0" sortType="ascending"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField axis="axisPage" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
-      <items count="10">
-        <item x="2"/>
-        <item x="1"/>
-        <item x="0"/>
-        <item m="1" x="7"/>
-        <item m="1" x="8"/>
-        <item m="1" x="3"/>
-        <item m="1" x="4"/>
-        <item m="1" x="5"/>
-        <item m="1" x="6"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="6"/>
-  </rowFields>
-  <rowItems count="4">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <pageFields count="4">
-    <pageField fld="7" hier="-1"/>
-    <pageField fld="1" hier="-1"/>
-    <pageField fld="18" hier="-1"/>
-    <pageField fld="10" hier="-1"/>
-  </pageFields>
-  <dataFields count="1">
-    <dataField name="Sum of Total amount in $" fld="12" baseField="16" baseItem="4"/>
-  </dataFields>
-  <formats count="2">
-    <format dxfId="36">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="37">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="16">
-    <chartFormat chart="2" format="6" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="2" format="7" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="2" format="8" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="3"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="2" format="9" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="6" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="6" format="1" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="6" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="3"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="9" format="6" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="9" format="7" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="9" format="8" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="3"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="12" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="12" format="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="17" format="6" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="17" format="7">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="17" format="8">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="17" format="9">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="3"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:Y501" totalsRowShown="0" headerRowDxfId="28" headerRowBorderDxfId="26" tableBorderDxfId="27" totalsRowBorderDxfId="25">
   <autoFilter ref="A1:Y501" xr:uid="{00000000-0009-0000-0100-000001000000}">
-    <filterColumn colId="8">
-      <filters>
-        <filter val="University of Malawi"/>
-      </filters>
-    </filterColumn>
     <filterColumn colId="18">
       <filters>
         <filter val="Graduate"/>
@@ -40330,7 +40328,7 @@
       <c r="X120" s="4"/>
       <c r="Y120" s="4"/>
     </row>
-    <row r="121" spans="1:25" hidden="1">
+    <row r="121" spans="1:25">
       <c r="A121" s="3">
         <v>120</v>
       </c>
@@ -43290,7 +43288,7 @@
       <c r="X167" s="4"/>
       <c r="Y167" s="4"/>
     </row>
-    <row r="168" spans="1:25" hidden="1">
+    <row r="168" spans="1:25">
       <c r="A168" s="3">
         <v>167</v>
       </c>
@@ -43352,7 +43350,7 @@
       <c r="X168" s="4"/>
       <c r="Y168" s="4"/>
     </row>
-    <row r="169" spans="1:25" hidden="1">
+    <row r="169" spans="1:25">
       <c r="A169" s="3">
         <v>168</v>
       </c>
@@ -43414,7 +43412,7 @@
       <c r="X169" s="4"/>
       <c r="Y169" s="4"/>
     </row>
-    <row r="170" spans="1:25" hidden="1">
+    <row r="170" spans="1:25">
       <c r="A170" s="3">
         <v>169</v>
       </c>
@@ -43476,7 +43474,7 @@
       <c r="X170" s="4"/>
       <c r="Y170" s="4"/>
     </row>
-    <row r="171" spans="1:25" hidden="1">
+    <row r="171" spans="1:25">
       <c r="A171" s="3">
         <v>170</v>
       </c>
@@ -43536,7 +43534,7 @@
       <c r="X171" s="4"/>
       <c r="Y171" s="4"/>
     </row>
-    <row r="172" spans="1:25" hidden="1">
+    <row r="172" spans="1:25">
       <c r="A172" s="3">
         <v>171</v>
       </c>
@@ -43598,7 +43596,7 @@
       <c r="X172" s="4"/>
       <c r="Y172" s="4"/>
     </row>
-    <row r="173" spans="1:25" hidden="1">
+    <row r="173" spans="1:25">
       <c r="A173" s="3">
         <v>172</v>
       </c>
@@ -43784,7 +43782,7 @@
       <c r="X175" s="4"/>
       <c r="Y175" s="4"/>
     </row>
-    <row r="176" spans="1:25" hidden="1">
+    <row r="176" spans="1:25">
       <c r="A176" s="3">
         <v>175</v>
       </c>
@@ -43842,7 +43840,7 @@
       <c r="X176" s="4"/>
       <c r="Y176" s="4"/>
     </row>
-    <row r="177" spans="1:25" hidden="1">
+    <row r="177" spans="1:25">
       <c r="A177" s="3">
         <v>176</v>
       </c>
@@ -43904,7 +43902,7 @@
       <c r="X177" s="4"/>
       <c r="Y177" s="4"/>
     </row>
-    <row r="178" spans="1:25" hidden="1">
+    <row r="178" spans="1:25">
       <c r="A178" s="3">
         <v>177</v>
       </c>
@@ -43966,7 +43964,7 @@
       <c r="X178" s="4"/>
       <c r="Y178" s="4"/>
     </row>
-    <row r="179" spans="1:25" hidden="1">
+    <row r="179" spans="1:25">
       <c r="A179" s="3">
         <v>178</v>
       </c>
@@ -44028,7 +44026,7 @@
       <c r="X179" s="4"/>
       <c r="Y179" s="4"/>
     </row>
-    <row r="180" spans="1:25" hidden="1">
+    <row r="180" spans="1:25">
       <c r="A180" s="3">
         <v>179</v>
       </c>
@@ -44090,7 +44088,7 @@
       <c r="X180" s="4"/>
       <c r="Y180" s="4"/>
     </row>
-    <row r="181" spans="1:25" hidden="1">
+    <row r="181" spans="1:25">
       <c r="A181" s="3">
         <v>180</v>
       </c>
@@ -44152,7 +44150,7 @@
       <c r="X181" s="4"/>
       <c r="Y181" s="4"/>
     </row>
-    <row r="182" spans="1:25" hidden="1">
+    <row r="182" spans="1:25">
       <c r="A182" s="3">
         <v>181</v>
       </c>
@@ -44214,7 +44212,7 @@
       <c r="X182" s="4"/>
       <c r="Y182" s="4"/>
     </row>
-    <row r="183" spans="1:25" hidden="1">
+    <row r="183" spans="1:25">
       <c r="A183" s="3">
         <v>182</v>
       </c>
@@ -44276,7 +44274,7 @@
       <c r="X183" s="4"/>
       <c r="Y183" s="4"/>
     </row>
-    <row r="184" spans="1:25" hidden="1">
+    <row r="184" spans="1:25">
       <c r="A184" s="3">
         <v>183</v>
       </c>
@@ -44338,7 +44336,7 @@
       <c r="X184" s="4"/>
       <c r="Y184" s="4"/>
     </row>
-    <row r="185" spans="1:25" hidden="1">
+    <row r="185" spans="1:25">
       <c r="A185" s="3">
         <v>184</v>
       </c>
@@ -44400,7 +44398,7 @@
       <c r="X185" s="4"/>
       <c r="Y185" s="4"/>
     </row>
-    <row r="186" spans="1:25" hidden="1">
+    <row r="186" spans="1:25">
       <c r="A186" s="3">
         <v>185</v>
       </c>
@@ -44456,7 +44454,7 @@
       <c r="X186" s="4"/>
       <c r="Y186" s="4"/>
     </row>
-    <row r="187" spans="1:25" hidden="1">
+    <row r="187" spans="1:25">
       <c r="A187" s="3">
         <v>186</v>
       </c>
@@ -44518,7 +44516,7 @@
       <c r="X187" s="4"/>
       <c r="Y187" s="4"/>
     </row>
-    <row r="188" spans="1:25" hidden="1">
+    <row r="188" spans="1:25">
       <c r="A188" s="3">
         <v>187</v>
       </c>
@@ -44580,7 +44578,7 @@
       <c r="X188" s="4"/>
       <c r="Y188" s="4"/>
     </row>
-    <row r="189" spans="1:25" hidden="1">
+    <row r="189" spans="1:25">
       <c r="A189" s="3">
         <v>188</v>
       </c>
@@ -44642,7 +44640,7 @@
       <c r="X189" s="4"/>
       <c r="Y189" s="4"/>
     </row>
-    <row r="190" spans="1:25" hidden="1">
+    <row r="190" spans="1:25">
       <c r="A190" s="3">
         <v>189</v>
       </c>
@@ -44704,7 +44702,7 @@
       <c r="X190" s="4"/>
       <c r="Y190" s="4"/>
     </row>
-    <row r="191" spans="1:25" hidden="1">
+    <row r="191" spans="1:25">
       <c r="A191" s="3">
         <v>190</v>
       </c>
@@ -44760,7 +44758,7 @@
       <c r="X191" s="4"/>
       <c r="Y191" s="4"/>
     </row>
-    <row r="192" spans="1:25" hidden="1">
+    <row r="192" spans="1:25">
       <c r="A192" s="3">
         <v>191</v>
       </c>
@@ -44818,7 +44816,7 @@
       <c r="X192" s="4"/>
       <c r="Y192" s="4"/>
     </row>
-    <row r="193" spans="1:25" hidden="1">
+    <row r="193" spans="1:25">
       <c r="A193" s="3">
         <v>192</v>
       </c>
@@ -44878,7 +44876,7 @@
       <c r="X193" s="4"/>
       <c r="Y193" s="4"/>
     </row>
-    <row r="194" spans="1:25" hidden="1">
+    <row r="194" spans="1:25">
       <c r="A194" s="3">
         <v>193</v>
       </c>
@@ -44936,7 +44934,7 @@
       <c r="X194" s="4"/>
       <c r="Y194" s="4"/>
     </row>
-    <row r="195" spans="1:25" hidden="1">
+    <row r="195" spans="1:25">
       <c r="A195" s="3">
         <v>194</v>
       </c>
@@ -44994,7 +44992,7 @@
       <c r="X195" s="4"/>
       <c r="Y195" s="4"/>
     </row>
-    <row r="196" spans="1:25" hidden="1">
+    <row r="196" spans="1:25">
       <c r="A196" s="3">
         <v>195</v>
       </c>
@@ -45052,7 +45050,7 @@
       <c r="X196" s="4"/>
       <c r="Y196" s="4"/>
     </row>
-    <row r="197" spans="1:25" hidden="1">
+    <row r="197" spans="1:25">
       <c r="A197" s="3">
         <v>196</v>
       </c>
@@ -45114,7 +45112,7 @@
       <c r="X197" s="4"/>
       <c r="Y197" s="4"/>
     </row>
-    <row r="198" spans="1:25" hidden="1">
+    <row r="198" spans="1:25">
       <c r="A198" s="3">
         <v>197</v>
       </c>
@@ -45174,7 +45172,7 @@
       <c r="X198" s="4"/>
       <c r="Y198" s="4"/>
     </row>
-    <row r="199" spans="1:25" hidden="1">
+    <row r="199" spans="1:25">
       <c r="A199" s="3">
         <v>198</v>
       </c>
@@ -45236,7 +45234,7 @@
       <c r="X199" s="4"/>
       <c r="Y199" s="4"/>
     </row>
-    <row r="200" spans="1:25" hidden="1">
+    <row r="200" spans="1:25">
       <c r="A200" s="3">
         <v>199</v>
       </c>
@@ -45296,7 +45294,7 @@
       <c r="X200" s="4"/>
       <c r="Y200" s="4"/>
     </row>
-    <row r="201" spans="1:25" hidden="1">
+    <row r="201" spans="1:25">
       <c r="A201" s="3">
         <v>200</v>
       </c>
@@ -45416,7 +45414,7 @@
       <c r="X202" s="4"/>
       <c r="Y202" s="4"/>
     </row>
-    <row r="203" spans="1:25" hidden="1">
+    <row r="203" spans="1:25">
       <c r="A203" s="3">
         <v>202</v>
       </c>
@@ -45476,7 +45474,7 @@
       <c r="X203" s="4"/>
       <c r="Y203" s="4"/>
     </row>
-    <row r="204" spans="1:25" hidden="1">
+    <row r="204" spans="1:25">
       <c r="A204" s="3">
         <v>203</v>
       </c>
@@ -45724,7 +45722,7 @@
       <c r="X207" s="4"/>
       <c r="Y207" s="4"/>
     </row>
-    <row r="208" spans="1:25" hidden="1">
+    <row r="208" spans="1:25">
       <c r="A208" s="3">
         <v>207</v>
       </c>
@@ -45786,7 +45784,7 @@
       <c r="X208" s="4"/>
       <c r="Y208" s="4"/>
     </row>
-    <row r="209" spans="1:25" hidden="1">
+    <row r="209" spans="1:25">
       <c r="A209" s="3">
         <v>208</v>
       </c>
@@ -45846,7 +45844,7 @@
       <c r="X209" s="4"/>
       <c r="Y209" s="4"/>
     </row>
-    <row r="210" spans="1:25" hidden="1">
+    <row r="210" spans="1:25">
       <c r="A210" s="3">
         <v>209</v>
       </c>
@@ -45906,7 +45904,7 @@
       <c r="X210" s="4"/>
       <c r="Y210" s="4"/>
     </row>
-    <row r="211" spans="1:25" hidden="1">
+    <row r="211" spans="1:25">
       <c r="A211" s="3">
         <v>210</v>
       </c>
@@ -45968,7 +45966,7 @@
       <c r="X211" s="4"/>
       <c r="Y211" s="4"/>
     </row>
-    <row r="212" spans="1:25" hidden="1">
+    <row r="212" spans="1:25">
       <c r="A212" s="3">
         <v>211</v>
       </c>
@@ -46030,7 +46028,7 @@
       <c r="X212" s="4"/>
       <c r="Y212" s="4"/>
     </row>
-    <row r="213" spans="1:25" hidden="1">
+    <row r="213" spans="1:25">
       <c r="A213" s="3">
         <v>212</v>
       </c>
@@ -46092,7 +46090,7 @@
       <c r="X213" s="4"/>
       <c r="Y213" s="4"/>
     </row>
-    <row r="214" spans="1:25" hidden="1">
+    <row r="214" spans="1:25">
       <c r="A214" s="3">
         <v>213</v>
       </c>
@@ -46154,7 +46152,7 @@
       <c r="X214" s="4"/>
       <c r="Y214" s="4"/>
     </row>
-    <row r="215" spans="1:25" hidden="1">
+    <row r="215" spans="1:25">
       <c r="A215" s="3">
         <v>214</v>
       </c>
@@ -46214,7 +46212,7 @@
       <c r="X215" s="4"/>
       <c r="Y215" s="4"/>
     </row>
-    <row r="216" spans="1:25" hidden="1">
+    <row r="216" spans="1:25">
       <c r="A216" s="3">
         <v>215</v>
       </c>
@@ -46274,7 +46272,7 @@
       <c r="X216" s="4"/>
       <c r="Y216" s="4"/>
     </row>
-    <row r="217" spans="1:25" hidden="1">
+    <row r="217" spans="1:25">
       <c r="A217" s="3">
         <v>216</v>
       </c>
@@ -46334,7 +46332,7 @@
       <c r="X217" s="4"/>
       <c r="Y217" s="4"/>
     </row>
-    <row r="218" spans="1:25" hidden="1">
+    <row r="218" spans="1:25">
       <c r="A218" s="3">
         <v>217</v>
       </c>
@@ -47600,7 +47598,7 @@
       <c r="X237" s="4"/>
       <c r="Y237" s="4"/>
     </row>
-    <row r="238" spans="1:25" hidden="1">
+    <row r="238" spans="1:25">
       <c r="A238" s="3">
         <v>237</v>
       </c>
@@ -47662,7 +47660,7 @@
       <c r="X238" s="4"/>
       <c r="Y238" s="4"/>
     </row>
-    <row r="239" spans="1:25" hidden="1">
+    <row r="239" spans="1:25">
       <c r="A239" s="3">
         <v>238</v>
       </c>
@@ -47724,7 +47722,7 @@
       <c r="X239" s="4"/>
       <c r="Y239" s="4"/>
     </row>
-    <row r="240" spans="1:25" hidden="1">
+    <row r="240" spans="1:25">
       <c r="A240" s="3">
         <v>239</v>
       </c>
@@ -47852,7 +47850,7 @@
       <c r="X241" s="4"/>
       <c r="Y241" s="4"/>
     </row>
-    <row r="242" spans="1:25" hidden="1">
+    <row r="242" spans="1:25">
       <c r="A242" s="3">
         <v>241</v>
       </c>
@@ -47982,7 +47980,7 @@
       <c r="X243" s="4"/>
       <c r="Y243" s="4"/>
     </row>
-    <row r="244" spans="1:25" hidden="1">
+    <row r="244" spans="1:25">
       <c r="A244" s="3">
         <v>243</v>
       </c>
@@ -48044,7 +48042,7 @@
       <c r="X244" s="4"/>
       <c r="Y244" s="4"/>
     </row>
-    <row r="245" spans="1:25" hidden="1">
+    <row r="245" spans="1:25">
       <c r="A245" s="3">
         <v>244</v>
       </c>
@@ -48104,7 +48102,7 @@
       <c r="X245" s="4"/>
       <c r="Y245" s="4"/>
     </row>
-    <row r="246" spans="1:25" hidden="1">
+    <row r="246" spans="1:25">
       <c r="A246" s="3">
         <v>245</v>
       </c>
@@ -48164,7 +48162,7 @@
       <c r="X246" s="4"/>
       <c r="Y246" s="4"/>
     </row>
-    <row r="247" spans="1:25" hidden="1">
+    <row r="247" spans="1:25">
       <c r="A247" s="3">
         <v>246</v>
       </c>
@@ -49742,7 +49740,7 @@
       <c r="X271" s="4"/>
       <c r="Y271" s="4"/>
     </row>
-    <row r="272" spans="1:25" hidden="1">
+    <row r="272" spans="1:25">
       <c r="A272" s="3">
         <v>271</v>
       </c>
@@ -49802,7 +49800,7 @@
       <c r="X272" s="4"/>
       <c r="Y272" s="4"/>
     </row>
-    <row r="273" spans="1:25" hidden="1">
+    <row r="273" spans="1:25">
       <c r="A273" s="3">
         <v>272</v>
       </c>
@@ -49866,7 +49864,7 @@
       <c r="X273" s="4"/>
       <c r="Y273" s="4"/>
     </row>
-    <row r="274" spans="1:25" hidden="1">
+    <row r="274" spans="1:25">
       <c r="A274" s="3">
         <v>273</v>
       </c>
@@ -49928,7 +49926,7 @@
       <c r="X274" s="4"/>
       <c r="Y274" s="4"/>
     </row>
-    <row r="275" spans="1:25" hidden="1">
+    <row r="275" spans="1:25">
       <c r="A275" s="3">
         <v>274</v>
       </c>
@@ -49988,7 +49986,7 @@
       <c r="X275" s="4"/>
       <c r="Y275" s="4"/>
     </row>
-    <row r="276" spans="1:25" hidden="1">
+    <row r="276" spans="1:25">
       <c r="A276" s="3">
         <v>275</v>
       </c>
@@ -50050,7 +50048,7 @@
       <c r="X276" s="4"/>
       <c r="Y276" s="4"/>
     </row>
-    <row r="277" spans="1:25" hidden="1">
+    <row r="277" spans="1:25">
       <c r="A277" s="3">
         <v>276</v>
       </c>
@@ -50176,7 +50174,7 @@
       <c r="X278" s="4"/>
       <c r="Y278" s="4"/>
     </row>
-    <row r="279" spans="1:25" hidden="1">
+    <row r="279" spans="1:25">
       <c r="A279" s="3">
         <v>278</v>
       </c>
@@ -50238,7 +50236,7 @@
       <c r="X279" s="4"/>
       <c r="Y279" s="4"/>
     </row>
-    <row r="280" spans="1:25" hidden="1">
+    <row r="280" spans="1:25">
       <c r="A280" s="3">
         <v>279</v>
       </c>
@@ -50302,7 +50300,7 @@
       <c r="X280" s="4"/>
       <c r="Y280" s="4"/>
     </row>
-    <row r="281" spans="1:25" hidden="1">
+    <row r="281" spans="1:25">
       <c r="A281" s="3">
         <v>280</v>
       </c>
@@ -51256,7 +51254,7 @@
       <c r="X295" s="4"/>
       <c r="Y295" s="4"/>
     </row>
-    <row r="296" spans="1:25" hidden="1">
+    <row r="296" spans="1:25">
       <c r="A296" s="3">
         <v>295</v>
       </c>
@@ -51320,7 +51318,7 @@
       <c r="X296" s="4"/>
       <c r="Y296" s="4"/>
     </row>
-    <row r="297" spans="1:25" hidden="1">
+    <row r="297" spans="1:25">
       <c r="A297" s="3">
         <v>296</v>
       </c>
@@ -51384,7 +51382,7 @@
       <c r="X297" s="4"/>
       <c r="Y297" s="4"/>
     </row>
-    <row r="298" spans="1:25" hidden="1">
+    <row r="298" spans="1:25">
       <c r="A298" s="3">
         <v>297</v>
       </c>
@@ -51512,7 +51510,7 @@
       <c r="X299" s="4"/>
       <c r="Y299" s="4"/>
     </row>
-    <row r="300" spans="1:25" hidden="1">
+    <row r="300" spans="1:25">
       <c r="A300" s="3">
         <v>299</v>
       </c>
@@ -51572,7 +51570,7 @@
       <c r="X300" s="4"/>
       <c r="Y300" s="4"/>
     </row>
-    <row r="301" spans="1:25" hidden="1">
+    <row r="301" spans="1:25">
       <c r="A301" s="3">
         <v>300</v>
       </c>
@@ -51634,7 +51632,7 @@
       <c r="X301" s="4"/>
       <c r="Y301" s="4"/>
     </row>
-    <row r="302" spans="1:25" hidden="1">
+    <row r="302" spans="1:25">
       <c r="A302" s="3">
         <v>301</v>
       </c>
@@ -51696,7 +51694,7 @@
       <c r="X302" s="4"/>
       <c r="Y302" s="4"/>
     </row>
-    <row r="303" spans="1:25" hidden="1">
+    <row r="303" spans="1:25">
       <c r="A303" s="3">
         <v>302</v>
       </c>
@@ -51764,7 +51762,7 @@
       <c r="X303" s="4"/>
       <c r="Y303" s="4"/>
     </row>
-    <row r="304" spans="1:25" hidden="1">
+    <row r="304" spans="1:25">
       <c r="A304" s="3">
         <v>303</v>
       </c>
@@ -51828,7 +51826,7 @@
       <c r="X304" s="4"/>
       <c r="Y304" s="4"/>
     </row>
-    <row r="305" spans="1:25" hidden="1">
+    <row r="305" spans="1:25">
       <c r="A305" s="3">
         <v>304</v>
       </c>
@@ -51892,7 +51890,7 @@
       <c r="X305" s="4"/>
       <c r="Y305" s="4"/>
     </row>
-    <row r="306" spans="1:25" hidden="1">
+    <row r="306" spans="1:25">
       <c r="A306" s="3">
         <v>305</v>
       </c>
@@ -52900,7 +52898,7 @@
       <c r="X320" s="4"/>
       <c r="Y320" s="4"/>
     </row>
-    <row r="321" spans="1:25" hidden="1">
+    <row r="321" spans="1:25">
       <c r="A321" s="3">
         <v>320</v>
       </c>
@@ -52960,7 +52958,7 @@
       <c r="X321" s="4"/>
       <c r="Y321" s="4"/>
     </row>
-    <row r="322" spans="1:25" hidden="1">
+    <row r="322" spans="1:25">
       <c r="A322" s="3">
         <v>321</v>
       </c>
@@ -53022,7 +53020,7 @@
       <c r="X322" s="4"/>
       <c r="Y322" s="4"/>
     </row>
-    <row r="323" spans="1:25" hidden="1">
+    <row r="323" spans="1:25">
       <c r="A323" s="3">
         <v>322</v>
       </c>
@@ -53084,7 +53082,7 @@
       <c r="X323" s="4"/>
       <c r="Y323" s="4"/>
     </row>
-    <row r="324" spans="1:25" hidden="1">
+    <row r="324" spans="1:25">
       <c r="A324" s="3">
         <v>323</v>
       </c>
@@ -53148,7 +53146,7 @@
       <c r="X324" s="4"/>
       <c r="Y324" s="4"/>
     </row>
-    <row r="325" spans="1:25" hidden="1">
+    <row r="325" spans="1:25">
       <c r="A325" s="3">
         <v>324</v>
       </c>
@@ -53202,7 +53200,7 @@
       <c r="X325" s="4"/>
       <c r="Y325" s="4"/>
     </row>
-    <row r="326" spans="1:25" hidden="1">
+    <row r="326" spans="1:25">
       <c r="A326" s="3">
         <v>325</v>
       </c>
@@ -53264,7 +53262,7 @@
       <c r="X326" s="4"/>
       <c r="Y326" s="4"/>
     </row>
-    <row r="327" spans="1:25" hidden="1">
+    <row r="327" spans="1:25">
       <c r="A327" s="3">
         <v>326</v>
       </c>
@@ -53382,7 +53380,7 @@
       <c r="X328" s="4"/>
       <c r="Y328" s="4"/>
     </row>
-    <row r="329" spans="1:25" ht="14.45" hidden="1" customHeight="1">
+    <row r="329" spans="1:25" ht="14.45" customHeight="1">
       <c r="A329" s="3">
         <v>328</v>
       </c>
@@ -54334,7 +54332,7 @@
       <c r="X342" s="4"/>
       <c r="Y342" s="4"/>
     </row>
-    <row r="343" spans="1:25" hidden="1">
+    <row r="343" spans="1:25">
       <c r="A343" s="3">
         <v>342</v>
       </c>
@@ -54398,7 +54396,7 @@
       <c r="X343" s="4"/>
       <c r="Y343" s="4"/>
     </row>
-    <row r="344" spans="1:25" hidden="1">
+    <row r="344" spans="1:25">
       <c r="A344" s="3">
         <v>343</v>
       </c>
@@ -54464,7 +54462,7 @@
       <c r="X344" s="4"/>
       <c r="Y344" s="4"/>
     </row>
-    <row r="345" spans="1:25" hidden="1">
+    <row r="345" spans="1:25">
       <c r="A345" s="3">
         <v>344</v>
       </c>
@@ -54526,7 +54524,7 @@
       <c r="X345" s="4"/>
       <c r="Y345" s="4"/>
     </row>
-    <row r="346" spans="1:25" hidden="1">
+    <row r="346" spans="1:25">
       <c r="A346" s="3">
         <v>345</v>
       </c>
@@ -54588,7 +54586,7 @@
       <c r="X346" s="4"/>
       <c r="Y346" s="4"/>
     </row>
-    <row r="347" spans="1:25" hidden="1">
+    <row r="347" spans="1:25">
       <c r="A347" s="3">
         <v>346</v>
       </c>
@@ -54728,7 +54726,7 @@
       <c r="X348" s="4"/>
       <c r="Y348" s="4"/>
     </row>
-    <row r="349" spans="1:25" hidden="1">
+    <row r="349" spans="1:25">
       <c r="A349" s="3">
         <v>348</v>
       </c>
@@ -54798,7 +54796,7 @@
       <c r="X349" s="4"/>
       <c r="Y349" s="4"/>
     </row>
-    <row r="350" spans="1:25" hidden="1">
+    <row r="350" spans="1:25">
       <c r="A350" s="3">
         <v>349</v>
       </c>
@@ -55826,7 +55824,7 @@
       <c r="X364" s="4"/>
       <c r="Y364" s="4"/>
     </row>
-    <row r="365" spans="1:25" hidden="1">
+    <row r="365" spans="1:25">
       <c r="A365" s="3">
         <v>364</v>
       </c>
@@ -55894,7 +55892,7 @@
       </c>
       <c r="Y365" s="4"/>
     </row>
-    <row r="366" spans="1:25" hidden="1">
+    <row r="366" spans="1:25">
       <c r="A366" s="3">
         <v>365</v>
       </c>
@@ -55964,7 +55962,7 @@
       </c>
       <c r="Y366" s="4"/>
     </row>
-    <row r="367" spans="1:25" hidden="1">
+    <row r="367" spans="1:25">
       <c r="A367" s="3">
         <v>366</v>
       </c>
@@ -56032,7 +56030,7 @@
       <c r="X367" s="4"/>
       <c r="Y367" s="4"/>
     </row>
-    <row r="368" spans="1:25" hidden="1">
+    <row r="368" spans="1:25">
       <c r="A368" s="3">
         <v>367</v>
       </c>
@@ -56094,7 +56092,7 @@
       </c>
       <c r="Y368" s="4"/>
     </row>
-    <row r="369" spans="1:25" hidden="1">
+    <row r="369" spans="1:25">
       <c r="A369" s="3">
         <v>368</v>
       </c>
@@ -56156,7 +56154,7 @@
       </c>
       <c r="Y369" s="4"/>
     </row>
-    <row r="370" spans="1:25" hidden="1">
+    <row r="370" spans="1:25">
       <c r="A370" s="3">
         <v>369</v>
       </c>
@@ -56226,7 +56224,7 @@
       </c>
       <c r="Y370" s="4"/>
     </row>
-    <row r="371" spans="1:25" hidden="1">
+    <row r="371" spans="1:25">
       <c r="A371" s="3">
         <v>370</v>
       </c>
@@ -56298,7 +56296,7 @@
       </c>
       <c r="Y371" s="4"/>
     </row>
-    <row r="372" spans="1:25" hidden="1">
+    <row r="372" spans="1:25">
       <c r="A372" s="3">
         <v>371</v>
       </c>
@@ -56368,7 +56366,7 @@
       </c>
       <c r="Y372" s="4"/>
     </row>
-    <row r="373" spans="1:25" hidden="1">
+    <row r="373" spans="1:25">
       <c r="A373" s="3">
         <v>372</v>
       </c>
@@ -56438,7 +56436,7 @@
       </c>
       <c r="Y373" s="4"/>
     </row>
-    <row r="374" spans="1:25" hidden="1">
+    <row r="374" spans="1:25">
       <c r="A374" s="3">
         <v>373</v>
       </c>
@@ -56508,7 +56506,7 @@
       </c>
       <c r="Y374" s="4"/>
     </row>
-    <row r="375" spans="1:25" hidden="1">
+    <row r="375" spans="1:25">
       <c r="A375" s="3">
         <v>374</v>
       </c>
@@ -56578,7 +56576,7 @@
       </c>
       <c r="Y375" s="4"/>
     </row>
-    <row r="376" spans="1:25" hidden="1">
+    <row r="376" spans="1:25">
       <c r="A376" s="3">
         <v>375</v>
       </c>
@@ -56650,7 +56648,7 @@
       </c>
       <c r="Y376" s="4"/>
     </row>
-    <row r="377" spans="1:25" hidden="1">
+    <row r="377" spans="1:25">
       <c r="A377" s="3">
         <v>376</v>
       </c>
@@ -56714,7 +56712,7 @@
       </c>
       <c r="Y377" s="4"/>
     </row>
-    <row r="378" spans="1:25" hidden="1">
+    <row r="378" spans="1:25">
       <c r="A378" s="3">
         <v>377</v>
       </c>
@@ -57322,7 +57320,7 @@
       <c r="X386" s="18"/>
       <c r="Y386" s="4"/>
     </row>
-    <row r="387" spans="1:25" hidden="1">
+    <row r="387" spans="1:25">
       <c r="A387" s="3">
         <v>386</v>
       </c>
@@ -57390,7 +57388,7 @@
       </c>
       <c r="Y387" s="4"/>
     </row>
-    <row r="388" spans="1:25" hidden="1">
+    <row r="388" spans="1:25">
       <c r="A388" s="3">
         <v>387</v>
       </c>
@@ -57458,7 +57456,7 @@
       </c>
       <c r="Y388" s="4"/>
     </row>
-    <row r="389" spans="1:25" hidden="1">
+    <row r="389" spans="1:25">
       <c r="A389" s="3">
         <v>388</v>
       </c>
@@ -57526,7 +57524,7 @@
       </c>
       <c r="Y389" s="4"/>
     </row>
-    <row r="390" spans="1:25" hidden="1">
+    <row r="390" spans="1:25">
       <c r="A390" s="3">
         <v>389</v>
       </c>
@@ -57588,7 +57586,7 @@
       <c r="X390" s="4"/>
       <c r="Y390" s="4"/>
     </row>
-    <row r="391" spans="1:25" hidden="1">
+    <row r="391" spans="1:25">
       <c r="A391" s="3">
         <v>390</v>
       </c>
@@ -57656,7 +57654,7 @@
       </c>
       <c r="Y391" s="4"/>
     </row>
-    <row r="392" spans="1:25" hidden="1">
+    <row r="392" spans="1:25">
       <c r="A392" s="3">
         <v>391</v>
       </c>
@@ -57780,7 +57778,7 @@
       </c>
       <c r="Y393" s="4"/>
     </row>
-    <row r="394" spans="1:25" hidden="1">
+    <row r="394" spans="1:25">
       <c r="A394" s="3">
         <v>393</v>
       </c>
@@ -57842,7 +57840,7 @@
       <c r="X394" s="3"/>
       <c r="Y394" s="4"/>
     </row>
-    <row r="395" spans="1:25" hidden="1">
+    <row r="395" spans="1:25">
       <c r="A395" s="3">
         <v>394</v>
       </c>
@@ -57908,7 +57906,7 @@
       </c>
       <c r="Y395" s="4"/>
     </row>
-    <row r="396" spans="1:25" hidden="1">
+    <row r="396" spans="1:25">
       <c r="A396" s="3">
         <v>395</v>
       </c>
@@ -58550,7 +58548,7 @@
       <c r="X405" s="3"/>
       <c r="Y405" s="4"/>
     </row>
-    <row r="406" spans="1:25" hidden="1">
+    <row r="406" spans="1:25">
       <c r="A406" s="3">
         <v>405</v>
       </c>
@@ -58616,7 +58614,7 @@
       </c>
       <c r="Y406" s="4"/>
     </row>
-    <row r="407" spans="1:25" hidden="1">
+    <row r="407" spans="1:25">
       <c r="A407" s="3">
         <v>406</v>
       </c>
@@ -58682,7 +58680,7 @@
       </c>
       <c r="Y407" s="4"/>
     </row>
-    <row r="408" spans="1:25" hidden="1">
+    <row r="408" spans="1:25">
       <c r="A408" s="3">
         <v>407</v>
       </c>
@@ -58750,7 +58748,7 @@
       </c>
       <c r="Y408" s="4"/>
     </row>
-    <row r="409" spans="1:25" hidden="1">
+    <row r="409" spans="1:25">
       <c r="A409" s="3">
         <v>408</v>
       </c>
@@ -58818,7 +58816,7 @@
       </c>
       <c r="Y409" s="4"/>
     </row>
-    <row r="410" spans="1:25" hidden="1">
+    <row r="410" spans="1:25">
       <c r="A410" s="3">
         <v>409</v>
       </c>
@@ -58952,7 +58950,7 @@
       </c>
       <c r="Y411" s="4"/>
     </row>
-    <row r="412" spans="1:25" hidden="1">
+    <row r="412" spans="1:25">
       <c r="A412" s="3">
         <v>411</v>
       </c>
@@ -59018,7 +59016,7 @@
       </c>
       <c r="Y412" s="4"/>
     </row>
-    <row r="413" spans="1:25" hidden="1">
+    <row r="413" spans="1:25">
       <c r="A413" s="3">
         <v>412</v>
       </c>
@@ -59086,7 +59084,7 @@
       </c>
       <c r="Y413" s="4"/>
     </row>
-    <row r="414" spans="1:25" hidden="1">
+    <row r="414" spans="1:25">
       <c r="A414" s="3">
         <v>413</v>
       </c>
@@ -59150,7 +59148,7 @@
       </c>
       <c r="Y414" s="4"/>
     </row>
-    <row r="415" spans="1:25" hidden="1">
+    <row r="415" spans="1:25">
       <c r="A415" s="3">
         <v>414</v>
       </c>
@@ -59210,7 +59208,7 @@
       <c r="X415" s="3"/>
       <c r="Y415" s="4"/>
     </row>
-    <row r="416" spans="1:25" hidden="1">
+    <row r="416" spans="1:25">
       <c r="A416" s="3">
         <v>415</v>
       </c>
@@ -59420,7 +59418,7 @@
       </c>
       <c r="Y418" s="4"/>
     </row>
-    <row r="419" spans="1:25" hidden="1">
+    <row r="419" spans="1:25">
       <c r="A419" s="3">
         <v>418</v>
       </c>
@@ -59488,7 +59486,7 @@
       <c r="X419" s="18"/>
       <c r="Y419" s="4"/>
     </row>
-    <row r="420" spans="1:25" hidden="1">
+    <row r="420" spans="1:25">
       <c r="A420" s="3">
         <v>419</v>
       </c>
@@ -59556,7 +59554,7 @@
       </c>
       <c r="Y420" s="4"/>
     </row>
-    <row r="421" spans="1:25" hidden="1">
+    <row r="421" spans="1:25">
       <c r="A421" s="3">
         <v>420</v>
       </c>
@@ -59626,7 +59624,7 @@
       </c>
       <c r="Y421" s="4"/>
     </row>
-    <row r="422" spans="1:25" hidden="1">
+    <row r="422" spans="1:25">
       <c r="A422" s="3">
         <v>421</v>
       </c>
@@ -59696,7 +59694,7 @@
       </c>
       <c r="Y422" s="4"/>
     </row>
-    <row r="423" spans="1:25" hidden="1">
+    <row r="423" spans="1:25">
       <c r="A423" s="3">
         <v>422</v>
       </c>
@@ -59766,7 +59764,7 @@
       </c>
       <c r="Y423" s="4"/>
     </row>
-    <row r="424" spans="1:25" hidden="1">
+    <row r="424" spans="1:25">
       <c r="A424" s="3">
         <v>423</v>
       </c>
@@ -59836,7 +59834,7 @@
       </c>
       <c r="Y424" s="4"/>
     </row>
-    <row r="425" spans="1:25" hidden="1">
+    <row r="425" spans="1:25">
       <c r="A425" s="3">
         <v>424</v>
       </c>
@@ -59906,7 +59904,7 @@
       </c>
       <c r="Y425" s="4"/>
     </row>
-    <row r="426" spans="1:25" hidden="1">
+    <row r="426" spans="1:25">
       <c r="A426" s="3">
         <v>425</v>
       </c>
@@ -59976,7 +59974,7 @@
       </c>
       <c r="Y426" s="4"/>
     </row>
-    <row r="427" spans="1:25" hidden="1">
+    <row r="427" spans="1:25">
       <c r="A427" s="3">
         <v>426</v>
       </c>
@@ -60046,7 +60044,7 @@
       </c>
       <c r="Y427" s="4"/>
     </row>
-    <row r="428" spans="1:25" hidden="1">
+    <row r="428" spans="1:25">
       <c r="A428" s="3">
         <v>427</v>
       </c>
@@ -60116,7 +60114,7 @@
       </c>
       <c r="Y428" s="4"/>
     </row>
-    <row r="429" spans="1:25" hidden="1">
+    <row r="429" spans="1:25">
       <c r="A429" s="3">
         <v>428</v>
       </c>
@@ -60316,7 +60314,7 @@
       </c>
       <c r="Y431" s="4"/>
     </row>
-    <row r="432" spans="1:25" hidden="1">
+    <row r="432" spans="1:25">
       <c r="A432" s="3">
         <v>431</v>
       </c>
@@ -60382,7 +60380,7 @@
       <c r="X432" s="4"/>
       <c r="Y432" s="4"/>
     </row>
-    <row r="433" spans="1:25" hidden="1">
+    <row r="433" spans="1:25">
       <c r="A433" s="3">
         <v>432</v>
       </c>
@@ -60506,7 +60504,7 @@
       <c r="X434" s="4"/>
       <c r="Y434" s="4"/>
     </row>
-    <row r="435" spans="1:25" hidden="1">
+    <row r="435" spans="1:25">
       <c r="A435" s="3">
         <v>434</v>
       </c>
@@ -60560,7 +60558,7 @@
       <c r="X435" s="4"/>
       <c r="Y435" s="4"/>
     </row>
-    <row r="436" spans="1:25" hidden="1">
+    <row r="436" spans="1:25">
       <c r="A436" s="3">
         <v>435</v>
       </c>
@@ -60624,7 +60622,7 @@
       <c r="X436" s="4"/>
       <c r="Y436" s="4"/>
     </row>
-    <row r="437" spans="1:25" hidden="1">
+    <row r="437" spans="1:25">
       <c r="A437" s="3">
         <v>436</v>
       </c>
@@ -60688,7 +60686,7 @@
       <c r="X437" s="4"/>
       <c r="Y437" s="4"/>
     </row>
-    <row r="438" spans="1:25" hidden="1">
+    <row r="438" spans="1:25">
       <c r="A438" s="3">
         <v>437</v>
       </c>
@@ -60752,7 +60750,7 @@
       <c r="X438" s="4"/>
       <c r="Y438" s="4"/>
     </row>
-    <row r="439" spans="1:25" hidden="1">
+    <row r="439" spans="1:25">
       <c r="A439" s="3">
         <v>438</v>
       </c>
@@ -60816,7 +60814,7 @@
       <c r="X439" s="4"/>
       <c r="Y439" s="4"/>
     </row>
-    <row r="440" spans="1:25" hidden="1">
+    <row r="440" spans="1:25">
       <c r="A440" s="3">
         <v>439</v>
       </c>
@@ -60880,7 +60878,7 @@
       <c r="X440" s="4"/>
       <c r="Y440" s="4"/>
     </row>
-    <row r="441" spans="1:25" hidden="1">
+    <row r="441" spans="1:25">
       <c r="A441" s="3">
         <v>440</v>
       </c>
@@ -60944,7 +60942,7 @@
       <c r="X441" s="4"/>
       <c r="Y441" s="4"/>
     </row>
-    <row r="442" spans="1:25" hidden="1">
+    <row r="442" spans="1:25">
       <c r="A442" s="3">
         <v>441</v>
       </c>
@@ -61008,7 +61006,7 @@
       <c r="X442" s="4"/>
       <c r="Y442" s="4"/>
     </row>
-    <row r="443" spans="1:25" hidden="1">
+    <row r="443" spans="1:25">
       <c r="A443" s="3">
         <v>442</v>
       </c>
@@ -61072,7 +61070,7 @@
       <c r="X443" s="18"/>
       <c r="Y443" s="4"/>
     </row>
-    <row r="444" spans="1:25" hidden="1">
+    <row r="444" spans="1:25">
       <c r="A444" s="3">
         <v>443</v>
       </c>
@@ -61140,7 +61138,7 @@
       </c>
       <c r="Y444" s="4"/>
     </row>
-    <row r="445" spans="1:25" hidden="1">
+    <row r="445" spans="1:25">
       <c r="A445" s="3">
         <v>444</v>
       </c>
@@ -61206,7 +61204,7 @@
       <c r="X445" s="18"/>
       <c r="Y445" s="4"/>
     </row>
-    <row r="446" spans="1:25" hidden="1">
+    <row r="446" spans="1:25">
       <c r="A446" s="3">
         <v>445</v>
       </c>
@@ -61536,7 +61534,7 @@
       <c r="X450" s="3"/>
       <c r="Y450" s="4"/>
     </row>
-    <row r="451" spans="1:25" hidden="1">
+    <row r="451" spans="1:25">
       <c r="A451" s="3">
         <v>451</v>
       </c>
@@ -61602,7 +61600,7 @@
       <c r="X451" s="3"/>
       <c r="Y451" s="4"/>
     </row>
-    <row r="452" spans="1:25" hidden="1">
+    <row r="452" spans="1:25">
       <c r="A452" s="3">
         <v>452</v>
       </c>
@@ -61670,7 +61668,7 @@
       </c>
       <c r="Y452" s="4"/>
     </row>
-    <row r="453" spans="1:25" hidden="1">
+    <row r="453" spans="1:25">
       <c r="A453" s="3">
         <v>453</v>
       </c>
@@ -61726,7 +61724,7 @@
       <c r="X453" s="3"/>
       <c r="Y453" s="4"/>
     </row>
-    <row r="454" spans="1:25" hidden="1">
+    <row r="454" spans="1:25">
       <c r="A454" s="3">
         <v>454</v>
       </c>
@@ -61794,7 +61792,7 @@
       </c>
       <c r="Y454" s="4"/>
     </row>
-    <row r="455" spans="1:25" hidden="1">
+    <row r="455" spans="1:25">
       <c r="A455" s="3">
         <v>455</v>
       </c>
@@ -61856,7 +61854,7 @@
       </c>
       <c r="Y455" s="4"/>
     </row>
-    <row r="456" spans="1:25" hidden="1">
+    <row r="456" spans="1:25">
       <c r="A456" s="3">
         <v>456</v>
       </c>
@@ -61920,7 +61918,7 @@
       </c>
       <c r="Y456" s="4"/>
     </row>
-    <row r="457" spans="1:25" hidden="1">
+    <row r="457" spans="1:25">
       <c r="A457" s="3">
         <v>457</v>
       </c>
@@ -61986,7 +61984,7 @@
       </c>
       <c r="Y457" s="4"/>
     </row>
-    <row r="458" spans="1:25" hidden="1">
+    <row r="458" spans="1:25">
       <c r="A458" s="3">
         <v>458</v>
       </c>
@@ -62050,7 +62048,7 @@
       </c>
       <c r="Y458" s="4"/>
     </row>
-    <row r="459" spans="1:25" hidden="1">
+    <row r="459" spans="1:25">
       <c r="A459" s="3">
         <v>459</v>
       </c>
@@ -62118,7 +62116,7 @@
       </c>
       <c r="Y459" s="4"/>
     </row>
-    <row r="460" spans="1:25" hidden="1">
+    <row r="460" spans="1:25">
       <c r="A460" s="3">
         <v>460</v>
       </c>
@@ -62182,7 +62180,7 @@
       </c>
       <c r="Y460" s="4"/>
     </row>
-    <row r="461" spans="1:25" hidden="1">
+    <row r="461" spans="1:25">
       <c r="A461" s="3">
         <v>461</v>
       </c>
@@ -62248,7 +62246,7 @@
       <c r="X461" s="18"/>
       <c r="Y461" s="4"/>
     </row>
-    <row r="462" spans="1:25" hidden="1">
+    <row r="462" spans="1:25">
       <c r="A462" s="3">
         <v>462</v>
       </c>
@@ -62318,7 +62316,7 @@
       <c r="X462" s="18"/>
       <c r="Y462" s="4"/>
     </row>
-    <row r="463" spans="1:25" hidden="1">
+    <row r="463" spans="1:25">
       <c r="A463" s="3">
         <v>463</v>
       </c>
@@ -62386,7 +62384,7 @@
       <c r="X463" s="18"/>
       <c r="Y463" s="4"/>
     </row>
-    <row r="464" spans="1:25" hidden="1">
+    <row r="464" spans="1:25">
       <c r="A464" s="3">
         <v>464</v>
       </c>
@@ -62454,7 +62452,7 @@
       <c r="X464" s="4"/>
       <c r="Y464" s="4"/>
     </row>
-    <row r="465" spans="1:25" ht="12.75" hidden="1" customHeight="1">
+    <row r="465" spans="1:25" ht="12.75" customHeight="1">
       <c r="A465" s="3">
         <v>465</v>
       </c>
@@ -62518,7 +62516,7 @@
       </c>
       <c r="Y465" s="4"/>
     </row>
-    <row r="466" spans="1:25" hidden="1">
+    <row r="466" spans="1:25">
       <c r="A466" s="3">
         <v>466</v>
       </c>
@@ -62586,7 +62584,7 @@
       </c>
       <c r="Y466" s="4"/>
     </row>
-    <row r="467" spans="1:25" hidden="1">
+    <row r="467" spans="1:25">
       <c r="A467" s="3">
         <v>467</v>
       </c>
@@ -62726,7 +62724,7 @@
       </c>
       <c r="Y468" s="4"/>
     </row>
-    <row r="469" spans="1:25" hidden="1">
+    <row r="469" spans="1:25">
       <c r="A469" s="3">
         <v>469</v>
       </c>
@@ -62796,7 +62794,7 @@
       </c>
       <c r="Y469" s="4"/>
     </row>
-    <row r="470" spans="1:25" hidden="1">
+    <row r="470" spans="1:25">
       <c r="A470" s="3">
         <v>470</v>
       </c>
@@ -62860,7 +62858,7 @@
       <c r="X470" s="18"/>
       <c r="Y470" s="4"/>
     </row>
-    <row r="471" spans="1:25" hidden="1">
+    <row r="471" spans="1:25">
       <c r="A471" s="3">
         <v>471</v>
       </c>
@@ -63132,7 +63130,7 @@
       </c>
       <c r="Y474" s="4"/>
     </row>
-    <row r="475" spans="1:25" hidden="1">
+    <row r="475" spans="1:25">
       <c r="A475" s="3">
         <v>475</v>
       </c>
@@ -63198,7 +63196,7 @@
       </c>
       <c r="Y475" s="4"/>
     </row>
-    <row r="476" spans="1:25" hidden="1">
+    <row r="476" spans="1:25">
       <c r="A476" s="3">
         <v>476</v>
       </c>
@@ -63268,7 +63266,7 @@
       </c>
       <c r="Y476" s="4"/>
     </row>
-    <row r="477" spans="1:25" hidden="1">
+    <row r="477" spans="1:25">
       <c r="A477" s="3">
         <v>477</v>
       </c>
@@ -63336,7 +63334,7 @@
       </c>
       <c r="Y477" s="4"/>
     </row>
-    <row r="478" spans="1:25" hidden="1">
+    <row r="478" spans="1:25">
       <c r="A478" s="3">
         <v>478</v>
       </c>
@@ -63546,7 +63544,7 @@
       <c r="X480" s="57"/>
       <c r="Y480" s="18"/>
     </row>
-    <row r="481" spans="1:25" hidden="1">
+    <row r="481" spans="1:25">
       <c r="A481" s="3">
         <v>481</v>
       </c>
@@ -63616,7 +63614,7 @@
       </c>
       <c r="Y481" s="4"/>
     </row>
-    <row r="482" spans="1:25" hidden="1">
+    <row r="482" spans="1:25">
       <c r="A482" s="3">
         <v>482</v>
       </c>
@@ -63684,7 +63682,7 @@
       </c>
       <c r="Y482" s="4"/>
     </row>
-    <row r="483" spans="1:25" hidden="1">
+    <row r="483" spans="1:25">
       <c r="A483" s="3">
         <v>483</v>
       </c>
@@ -63750,7 +63748,7 @@
       </c>
       <c r="Y483" s="4"/>
     </row>
-    <row r="484" spans="1:25" hidden="1">
+    <row r="484" spans="1:25">
       <c r="A484" s="3">
         <v>484</v>
       </c>
@@ -63818,7 +63816,7 @@
       <c r="X484" s="3"/>
       <c r="Y484" s="4"/>
     </row>
-    <row r="485" spans="1:25" hidden="1">
+    <row r="485" spans="1:25">
       <c r="A485" s="3">
         <v>485</v>
       </c>
@@ -63884,7 +63882,7 @@
       </c>
       <c r="Y485" s="4"/>
     </row>
-    <row r="486" spans="1:25" hidden="1">
+    <row r="486" spans="1:25">
       <c r="A486" s="3">
         <v>486</v>
       </c>
@@ -63954,7 +63952,7 @@
       </c>
       <c r="Y486" s="4"/>
     </row>
-    <row r="487" spans="1:25" hidden="1">
+    <row r="487" spans="1:25">
       <c r="A487" s="3">
         <v>487</v>
       </c>
@@ -64022,7 +64020,7 @@
       </c>
       <c r="Y487" s="4"/>
     </row>
-    <row r="488" spans="1:25" hidden="1">
+    <row r="488" spans="1:25">
       <c r="A488" s="3">
         <v>488</v>
       </c>
@@ -64088,7 +64086,7 @@
       </c>
       <c r="Y488" s="4"/>
     </row>
-    <row r="489" spans="1:25" hidden="1">
+    <row r="489" spans="1:25">
       <c r="A489" s="3">
         <v>489</v>
       </c>
@@ -64154,7 +64152,7 @@
       </c>
       <c r="Y489" s="4"/>
     </row>
-    <row r="490" spans="1:25" hidden="1">
+    <row r="490" spans="1:25">
       <c r="A490" s="3">
         <v>490</v>
       </c>
@@ -64224,7 +64222,7 @@
       </c>
       <c r="Y490" s="18"/>
     </row>
-    <row r="491" spans="1:25" hidden="1">
+    <row r="491" spans="1:25">
       <c r="A491" s="3">
         <v>491</v>
       </c>
@@ -64292,7 +64290,7 @@
       </c>
       <c r="Y491" s="4"/>
     </row>
-    <row r="492" spans="1:25" hidden="1">
+    <row r="492" spans="1:25">
       <c r="A492" s="3">
         <v>492</v>
       </c>
@@ -64360,7 +64358,7 @@
       </c>
       <c r="Y492" s="4"/>
     </row>
-    <row r="493" spans="1:25" hidden="1">
+    <row r="493" spans="1:25">
       <c r="A493" s="3">
         <v>493</v>
       </c>
@@ -64496,7 +64494,7 @@
       </c>
       <c r="Y494" s="4"/>
     </row>
-    <row r="495" spans="1:25" hidden="1">
+    <row r="495" spans="1:25">
       <c r="A495" s="3">
         <v>495</v>
       </c>
@@ -64564,7 +64562,7 @@
       </c>
       <c r="Y495" s="18"/>
     </row>
-    <row r="496" spans="1:25" hidden="1">
+    <row r="496" spans="1:25">
       <c r="A496" s="3">
         <v>496</v>
       </c>
@@ -64914,7 +64912,7 @@
       </c>
       <c r="Y500" s="18"/>
     </row>
-    <row r="501" spans="1:25" hidden="1">
+    <row r="501" spans="1:25">
       <c r="A501" s="3">
         <v>501</v>
       </c>

</xml_diff>